<commit_message>
Add lot2plus, maintenance, and analysis tabs to Program_Spec_Combined.xlsx
Adds the three new protocol-derived spec tabs as sheets in the combined
Excel workbook, matching the existing column layout and formatting:
- lot2plus (16 rows): LOT2-5 classification, start/end rules, 30-day window
- maintenance (23 rows): valid therapies, 120-day rule, post-SCT rules
- analysis (10 rows): descriptive analysis plan, sensitivity, QC/validation

Workbook now has 10 tabs (was 7).

https://claude.ai/code/session_01YPW7e44rEGvrYNbVpdVpMn
</commit_message>
<xml_diff>
--- a/docs/Part 3/Program Spec/Program_Spec_Combined.xlsx
+++ b/docs/Part 3/Program Spec/Program_Spec_Combined.xlsx
@@ -14,6 +14,9 @@
     <sheet name="mma-med" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="sct" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="studypoppage" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="lot2plus" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="maintenance" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="analysis" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -52,8 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -544,7 +550,6 @@
           <t>Original spec had garbled text ('ID_PD end at ends at') and omitted health plan disenrollment as a follow-up endpoint. Protocol and code both correctly include death, disenrollment, and study end.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Original said 'ID_PD end at ends at the earliest of death or the end of the study period' which was garbled text and omitted health plan disenrollment as an endpoint.</t>
@@ -597,7 +602,6 @@
           <t>All three sources specify 01Jan2016 - 30June2025 consistently.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -650,7 +654,6 @@
           <t>All three sources agree: &gt;=1 inpatient (203.0x/C90.0x) or &gt;=2 outpatient within 90 days; earliest qualifying date = index date; 30/60 day flags for consideration.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -703,7 +706,6 @@
           <t>Original spec said 'medical OR pharmacy benefits'; protocol says 'medical AND pharmacy benefits'. Code uses T_MEMBER_CONT_ENROLLMENT which per Optum CDM Section 4.4 restricts to members with both medical and pharmacy benefits, so code aligns with protocol.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>Original program spec said 'medical or pharmacy benefits'. Protocol (Section 4.2, Criterion 3) states 'medical and pharmacy benefits'. Changed 'or' to 'and'.</t>
@@ -756,7 +758,6 @@
           <t>Original spec defined FU as 'from index date til end of patient identification period' - omitting death and disenrollment as endpoints. Protocol specifies earliest of death/disenrollment/study end. Code correctly implements ENDDATE_CE = LEAST(study_end, DEATH_DT, disenrollment).</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Original definition said 'from the index date til the end of the patient identification period (inclusive)' which omitted death and health plan disenrollment as endpoints. Protocol (Section 4.2, Criterion 4) specifies the follow-up ends at the earliest of death, health plan disenrollment, or end of study period. Also added missing protocol language about patients with assigned date of death &lt;3 months being retained.</t>
@@ -809,7 +810,6 @@
           <t>All three sources use consistent day conversions: 6 months=183 days, 3 months=91 days. Protocol does not explicitly state conversion factors but all implementations are internally consistent.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>No discrepancy found. This is implementation-specific and not explicitly in the protocol.</t>
@@ -862,7 +862,6 @@
           <t>All three sources agree: smoldering MM patients are not excluded. Protocol Appendix C documents the pressure-testing rationale. Code implements non-diagnostic flags and keeps smoldering patients in the cohort.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>No discrepancy found. Consistent with protocol language in Section 4.2 regarding baseline criteria and Appendix C pressure-testing criteria.</t>
@@ -915,7 +914,6 @@
           <t>All three sources agree: &gt;=1 day CE required (not 6 months). 3-month CE flagged for sensitivity. Protocol Criterion 4 specifies &gt;=1 day. Code implements CE_f as 1-day check and CE_3mosf as sensitivity flag.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>No discrepancy found. The resolution aligns with protocol which requires &gt;=1 day of CE.</t>
@@ -968,7 +966,6 @@
           <t>All three sources agree on dual-approach inpatient classification (POS/TOS OR CONF_ID). Protocol does not detail the approach explicitly but requires inpatient claim identification; spec and code both implement the same OR logic per Optum business rules.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>No discrepancy found. Implementation-specific operational detail not explicitly in protocol but consistent with protocol intent regarding inpatient claim identification (Protocol Section 4.2, Inclusion Criterion 1).</t>
@@ -1021,7 +1018,6 @@
           <t>Not mentioned anywhere in original program spec PDF. Protocol Section 4.2 Inclusion Criterion 2 requires age &gt;= 18. Code implements this as a configurable inclusion criterion (default: apply_age=TRUE, min_age=18).</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.2, Inclusion Criterion 2) specifies 'Adults: &gt;= 18 years of age in index calendar year.' Code implements via AGE_INDEX_YR &gt;= 18.</t>
@@ -1074,7 +1070,6 @@
           <t>Not present as a dedicated criterion in original program spec. Protocol Section 4.2 Exclusion Criterion 1 explicitly defines this. Code implements as MM_bl_agents flag with attrition Step 4.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>Missing from original program spec as a standalone exclusion criterion. Protocol (Section 4.2, Exclusion Criterion 1) states: 'Evidence of an MM oncology therapy during the baseline period' as an explicit exclusion.</t>
@@ -1127,7 +1122,6 @@
           <t>Not in original program spec. Protocol specifies 60-day window for outpatient other cancer claims; code uses 30 days (more conservative). Protocol and code both implement the concept; window difference may be intentional. Default is currently OFF (apply_other_malig_excl=FALSE).</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.2, Exclusion Criterion 2) defines other cancer exclusion. Note: code uses 30-day window vs protocol's 60-day window - verify if intentional.</t>
@@ -1180,7 +1174,6 @@
           <t>Not in original program spec. Protocol Section 4.2 Exclusion Criterion 3 defines this. Code implements as PREGNANT_FLAG. Currently default OFF (apply_pregnancy_excl=FALSE).</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.2, Exclusion Criterion 3) specifies pregnancy exclusion covering baseline and follow-up periods.</t>
@@ -1233,7 +1226,6 @@
           <t>Not in original program spec. Protocol Section 4.2 lists this under Exclusion Criteria but as a flag. Code implements both baseline and follow-up flags. Currently default OFF (apply_clintrial_excl=FALSE).</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.2, Exclusion Criterion 4) specifies clinical trial participation flagging during baseline and follow-up periods.</t>
@@ -1286,7 +1278,6 @@
           <t>Not in original program spec as a standalone criterion. Protocol Section 4.2 requires evidence of MM treatment in follow-up and explicitly excludes corticosteroids-only as qualifying. Code implements as MM_FU_agents flag at attrition Step 3.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.2, Inclusion Criterion 5) requires evidence of MM oncology therapy during follow-up. Also states 'Receipt of corticosteroids only will not be considered evidence of receiving an approved MM oncology therapy.'</t>
@@ -1339,10 +1330,585 @@
           <t>Not in original program spec. Protocol Section 4.5 specifies death date = 15th of month. Code implements this with additional edge-case handling (same-month index date, year-only granularity, pre-index clamping) that goes beyond the protocol's simple rule.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>Missing from original program spec. Protocol (Section 4.5) states 'The assigned date of death for dataset construction is set to the 15th of the month.' Code implements this plus edge-case logic for same-month index dates and year-only mortality records.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Definition (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Additional Notes (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Optum CDM Implementation</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>R Code Implementation</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status (OrigSpec/Protocol/Code)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Date Modified (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>QC Reviewed (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Discrepancy Found in Original Program Spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Section 5.3 Overview</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>ANALYSIS_OVERVIEW</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Descriptive analysis overview</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Analyses will be descriptive and focused on (1) development and performance assessment of the claims-based LOT algorithm, (2) describe real-world treatment pathways/sequencing, and (3) sensitivity and subgroup analyses.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Data analysis: 'Overview Analyses will be descriptive and focused on (1) development and performance assessment of the claims-based LOT algorithm, (2) describe real-world treatment pathways/sequencing, and (3) sensitivity and subgroup analyses.'</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr"/>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>LOT Algorithm Assessment</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>LOT_DISTRIBUTION</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Distribution of number of LOTs per patient</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>The distribution of number of LOTs per patient and time between LOTs (mean, standard deviation, median, IQR, min, max) will be tabulated. The most frequent regimens observed in LOT1, LOT2 and subsequent LOTs will be reported with counts and percentages.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 1: 'The distribution of number of LOTs per patient and time between LOTs (mean, standard deviation, median, IQR, min, max) will be tabulated. The most frequent regimens observed in LOT1, LOT2 and subsequent LOTs will be reported with counts and percentages.'</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LOT Algorithm Assessment</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>LOT_ANALYSIS_DATASET</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Per-LOT analysis dataset contents</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>For each LOT, the analysis datasets will include LOT start and end dates, agents/regimens present, and indicators for receipt of CAR-T, type of SCT, and maintenance therapy, as appropriate.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 1: 'For each LOT, the analysis datasets will include LOT start and end dates, agents/regimens present, and indicators for receipt of CAR-T, type of SCT, and maintenance therapy, as appropriate.'</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Treatment Pathways</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>TREATMENT_PATHWAYS</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Descriptive analyses of treatment pathways</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Treatment pathways will be described using sequence summaries and visualizations (e.g., Sankey plots) showing transitions across regimen classes and LOTs.</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 2: 'Treatment pathways will be described using sequence summaries and visualizations (e.g., Sankey plots) showing transitions across regimen classes and LOTs.'</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Treatment Pathways</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>INTERVENTION_UTILIZATION</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Utilization of key interventions</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Utilization of key interventions (SCT, CAR-T) and use of maintenance therapy will be reported as counts (n, %) and descriptively (median [IQR], mean [SD]).</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 2: 'Utilization of key interventions (SCT, CAR-T, enrollment codes for clinical trials where identifiable) and use of maintenance therapy will be reported as counts (n, %) and descriptively (median [IQR], mean [SD]).'</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity Analyses</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>SENSITIVITY_CE_VARIATION</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity: varying CE requirements</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters (e.g., required amount of continuous enrollment in the follow up period, look-back windows for prior exposure).</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 3: 'Sensitivity analyses will assess robustness of LOT rules by varying key algorithm parameters (e.g., required amount of continuous enrollment in the follow up period, inclusion/exclusion of corticosteroid-only claims, look-back windows for prior exposure).'</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr"/>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity Analyses</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>SENSITIVITY_COHORT_DEFS</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity: alternative cohort definitions</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity analyses applying alternative cohort definitions (e.g., applying varying patient identification criterion, stricter continuous enrollment criteria, varying eligibility criteria to the starting patient population).</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 3: 'applying alternative cohort definitions (e.g., applying varying patient identification criterion, stricter continuous enrollment criteria, varying eligibility criteria to the starting patient population [as listed in Section 4.2]).'</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr"/>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity Analyses</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>SENSITIVITY_OUTPUTS</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Sensitivity: effects on primary outputs</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Effects on primary outputs (number of LOTs, timing, regimen classification) will be reported.</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Item 3: 'Effects on primary outputs (number of LOTs, timing, regimen classification) will be reported.'</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="inlineStr"/>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>QC and Validation</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>LOT_VALIDATION</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>LOT algorithm validation</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Validation of the LOT algorithm will include clinical adjudication and comparing the finalized LOT to external benchmarks. These benchmarks include claims-derived treatment sequences, regimen frequencies and LOT distributions. Outputs will be compared to published LOT definitions and registry data, where available. Descriptive comparisons and standardized differences will be reviewed by the study team.</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3.1 Quality Control and Quality Assurance: 'Validation of the LOT algorithm will include clinical adjudication and comparing the finalized LOT to external benchmarks. These benchmarks include claims-derived treatment sequences, regimen frequencies and LOT distributions. Outputs will be compared to published LOT definitions and registry data, where available. Descriptive comparisons and standardized differences will be reviewed by the study team.'</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for analysis plan</t>
         </is>
       </c>
     </row>
@@ -1482,8 +2048,6 @@
           <t>Spec=Y: matches protocol definition. Protocol=Y: correctly defines observation end. Code=N: Code uses OBS_END_DT (coalesce of ENDDATE_CE and ENDDATE) rather than raw ENDDATE. This is a refinement - ENDDATE_CE properly accounts for disenrollment gaps while ENDDATE may extend beyond disenrollment. The code is more conservative/correct than the spec's simple ENDDATE reference.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>Minor discrepancy: Spec says 'merge ENDDATE from ELIG_COH' but the R code actually uses OBS_END_DT = coalesce(ENDDATE_CE, ENDDATE) which is more precise. ENDDATE_CE incorporates disenrollment end dates. This is a deliberate code improvement over the spec but creates a spec-code mismatch.</t>
@@ -1536,8 +2100,6 @@
           <t>Spec=Y: Correctly defines LOT1_START_DT as min(MAP_START_DT) where MAP_MED_CLASS != STEROID. Protocol=Y: Matches Section 5.1.1 LOT start definition. Code=Y: Implements exact same logic at line 3321-3323.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1590,8 +2152,6 @@
           <t>Spec=Y: 60-day window (LOT1_START_DT+59) matches protocol. Protocol=Y: Section 5.1.1 specifies 60 days for LOT1 regimen. Code=Y: induction_window_days=60, date_add(LOT1_START_DT, 59) implements days 0-59 = 60 days.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1644,8 +2204,6 @@
           <t>Spec=Y: Correctly defined as sum of LOT1_MED_[MED] flags. Protocol=Y: Consistent with regimen definition. Code=Y: Uses count(DISTINCT MED_ABBR) which is equivalent.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1698,8 +2256,6 @@
           <t>Spec=Y: Correctly derives class flags from med flags via CL_MMA_ROLLUP. Protocol=Y: Drug class categorization consistent with NCCN/FDA classifications. Code=Y: Implements via max(case when MED_CLASS=...) which is equivalent.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1752,8 +2308,6 @@
           <t>Spec=Y: Correctly defines discon as max MAP_END_DT with 90-day gap confirmation and permissible subs. Protocol=Y: Matches discontinuation definition in Section 5.1.1. Code=Y: Implements all three components (base meds + permissible subs, max MAP_END_DT, 90-day gap check).</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol. The spec's 90-day threshold for setting discon to missing is correctly implemented in code using cfg$lot_discon_gap_days=90.</t>
@@ -1806,8 +2360,6 @@
           <t>Spec=Y: Correctly defines as string of medication abbreviations. Protocol=Y: Consistent with regimen identification. Code=Y: Implements with sort_array(collect_set()) for deterministic ordering.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -1860,8 +2412,6 @@
           <t>Spec=N: Spec only considers two cases (discon_dt present or missing). Protocol=Y: LOT end includes medication add as a terminating event. Code=Y: Correctly handles three cases: (1) add-med ends base before discon, (2) discon ends base, (3) fallback to OBS_END_DT.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>Discrepancy: The spec defines LOT1_BASE_LENGTH with only two branches (discon present vs missing) but does not account for the LOT1_BASE_1ST_ADD_MED_DT case. The R code correctly adds a third branch: if a new medication is added (LOT1_BASE_1ST_ADD_MED_DT) before discontinuation, the base period ends at the add-med date. This is consistent with the protocol (Section 5.1.1 item 1: substitution of a new MM treatment ends the LOT). The spec is incomplete.</t>
@@ -1914,8 +2464,6 @@
           <t>Spec=Y: Correctly defines as day before earliest non-base-med MAP. Protocol=Y: Matches Section 5.1.1 new agent rule. Code=N (minor): Code uses min(MAP_MED_TYPE) for same-day ties instead of random selection as spec states. This is a deliberate, documented deviation for reproducibility.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>Minor discrepancy: Spec states 'select one of them at random' for same-day ties. Code uses min(MAP_MED_TYPE) instead for deterministic results (documented at line 3435). The MAP_MED_TYPE selection only affects LOT1_BASE_1ST_ADD_MED name, not the date. This is a reasonable implementation choice for reproducibility.</t>
@@ -1968,8 +2516,6 @@
           <t>Spec=Y: Correctly defined as medication name from add-med logic. Protocol=Y: Implicit in LOT transition rules. Code=N (minor): Uses min() instead of random for tie-breaking, same as LOT1_BASE_1ST_ADD_MED_DT deviation.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>Minor discrepancy: Same tie-breaking deviation as LOT1_BASE_1ST_ADD_MED_DT - code uses min() instead of random. See LOT1_BASE_1ST_ADD_MED_DT row for details.</t>
@@ -2022,8 +2568,6 @@
           <t>Spec=missing: The lot1base spec does not mention mesna exclusion. Protocol=Y: Explicitly states mesna is excluded. Code=Y: Mesna absent from codelists so implicitly excluded.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1.1 explicitly excludes mesna from LOTs but the lot1base program specification does not mention this rule. While mesna is implicitly excluded by not being in the codelist, the spec should document this exclusion for completeness.</t>
@@ -2076,8 +2620,6 @@
           <t>Spec=missing: lot1base spec does not document the 28-day assumption. Protocol=Y: Explicitly states 28-day default. Code=Y: Implements via cfg$medical_day_supply=28.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol explicitly defines the 28-day default for medical claims days supply and anomalous pharmacy claims, but the lot1base spec does not document this assumption. This is critical for understanding how LOT1_BASE_DISCON_DT is calculated.</t>
@@ -2130,8 +2672,6 @@
           <t>Spec=missing: lot1base spec references MAP_STACKED but does not document the pushout rule that generates it. Protocol=Y: Explicitly describes pushout. Code=Y: MAP algorithm implements pushout correctly per protocol.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>Missing from spec: The lot1base spec references MAP_STACKED dataset but does not document how overlapping pharmacy prescriptions push out run-out dates. This is defined in the MAP_MED spec (5B) but should be cross-referenced in lot1base for completeness since it directly affects LOT1_BASE_DISCON_DT.</t>
@@ -2184,8 +2724,6 @@
           <t>Spec=missing: lot1base spec does not explicitly clarify the dual role of steroids (excluded from start, included in regimen). Protocol=Y: Clear distinction. Code=Y: Correctly implements both exclusion from start and inclusion in regimen.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>Missing from spec: The lot1base spec does not explicitly document that steroids are excluded from LOT1_START_DT determination but included in induction regimen identification. Protocol Sections 4.2 and 5.1 make this distinction clear. The code correctly handles this but the spec should document this nuance.</t>
@@ -2238,8 +2776,6 @@
           <t>Spec=missing: lot1base spec does not mention the 60-day SCT window rule. Protocol=Y: Explicitly states 60-day rule with clinical rationale. Code=Y: cfg$sct_auto_gap_days=60 implements this.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1.1 defines a critical rule that SCTs must occur within 60 days of induction/maintenance end to remain part of LOT1. The lot1base spec does not reference this rule. It may be in the SCT spec (sct.pdf) but should be cross-referenced here since it affects LOT1 continuity.</t>
@@ -2292,8 +2828,6 @@
           <t>Spec=missing: lot1base spec does not define tandem SCT rules. Protocol=Y: Explicit 60-180 day window. Code=Y: Implements via cfg$sct_tandem_days=180 and tandem detection logic.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol defines planned tandem SCT (2 autologous SCTs 60-180 days apart) as a continuation of LOT1, but the lot1base spec does not mention this. May be covered in sct.pdf but should be cross-referenced here.</t>
@@ -2346,8 +2880,6 @@
           <t>Spec=missing: lot1base spec does not document unplanned SCT LOT termination rules. Protocol=Y: Explicit rules for unplanned AUTO and ALLO ending LOT. Code=Y: Implements full priority logic (AUTO excess, ALLO, CART).</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Sections 5.1 and 5.1.1 define critical rules about when SCTs end LOT1 (unplanned AUTO &gt; 180 days, any ALLO). The lot1base spec does not document these. These are likely in sct.pdf/lot1baseend.pdf but should be cross-referenced here since they determine LOT1 end.</t>
@@ -2400,8 +2932,6 @@
           <t>Spec=missing: lot1base spec does not mention CAR-T LOT classification. Protocol=Y: Explicit CAR-T rules in Section 5.1.2. Code=Y: CAR-T ends LOT1 and is tracked as separate LOT.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1.2 defines CAR-T as its own LOT with a 30-day consolidation window. The lot1base spec does not document this. The code implements CAR-T as a LOT1 terminator but the CAR-T LOT classification itself is a downstream concept.</t>
@@ -2454,8 +2984,6 @@
           <t>Spec=missing: lot1base spec does not define maintenance transition rules. Protocol=Y: Detailed maintenance rules in Section 5.1. Code=partial: Structural support exists but not fully integrated. Code comment explicitly notes maintenance specs not yet provided.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1 defines detailed maintenance regimen rules (120-day period, valid therapies, 30-day post-SCT variant) that can end LOT1 BASE. The lot1base spec does not document this. The R code notes at lines 4037-4038 that maintenance is not yet fully implemented, creating a protocol-code gap as well.</t>
@@ -2508,8 +3036,6 @@
           <t>Spec=missing: lot1base spec does not define LOT1_BASE_END_REASON. Protocol=Y: Lists all LOT end conditions. Code=Y: Implements full priority chain with categorical reason codes.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>Missing from spec: The lot1base program spec does not include LOT1_BASE_END_REASON as a variable, but it is implemented in the R code and is essential for understanding why LOT1 ended. Protocol Section 5.1.1 lists all end conditions. This variable should be added to the spec. It may be defined in lot1baseend.pdf instead.</t>
@@ -2562,8 +3088,6 @@
           <t>Spec=missing: lot1base spec does not define LOT1_BASE_END_DT (it only has LOT1_BASE_DISCON_DT and LOT1_BASE_1ST_ADD_MED_DT as separate variables). Protocol=Y: Implicit from LOT end rules. Code=Y: Implements as LOT1_BASE_END_DT in lot1_base_end view.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>Missing from spec: The lot1base spec defines LOT1_BASE_DISCON_DT and LOT1_BASE_1ST_ADD_MED_DT separately but does not define a unified LOT1_BASE_END_DT that combines all end conditions (including SCT). This is implemented in the R code. It may be defined in lot1baseend.pdf instead.</t>
@@ -2616,8 +3140,6 @@
           <t>Spec=missing: lot1base spec does not mention this rule. Protocol=Y: Explicitly defined as LOT end condition item 4. Code=partial: SCT detection exists but maintenance follow-up check not yet integrated.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1.1 item 4 defines that SCT without maintenance within 180 days ends the LOT at the SCT date. The lot1base spec omits this. The R code has not yet fully implemented this rule (maintenance specs noted as pending at lines 4037-4038).</t>
@@ -2670,8 +3192,6 @@
           <t>Spec=missing: lot1base spec does not describe the allogeneic SCT creating its own LOT. Protocol=Y: Explicitly defined. Code=Y: ALLO ends LOT1 and is tracked for downstream LOT creation.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>Missing from spec: Protocol Section 5.1 defines that allogeneic SCT creates its own LOT consisting entirely of the SCT with no other MM therapies. The lot1base spec does not document this. While the new LOT creation is downstream of LOT1_BASE, the LOT1 termination and characterization should be documented here.</t>
@@ -2724,8 +3244,6 @@
           <t>Spec=missing: lot1base spec does not include the overarching LOT1 classification definition from the protocol. Protocol=Y: Section 5.1.2 provides clear definition. Code=Y: Implementation spans multiple steps covering induction, SCT, and partial maintenance.</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>Missing from spec: The lot1base spec jumps into variable definitions without stating the overarching LOT1 classification from Protocol Section 5.1.2: that LOT1 includes induction and may include maintenance and SCTs. This framing context should be included to orient the reader.</t>
@@ -2778,8 +3296,6 @@
           <t>Spec=N: Spec mentions permissible substitutions in Additional Notes but does not provide a complete enumerable list. Protocol=Y: Lists all four categories explicitly. Code=Y: Implements via permissible_subs table and codelist mapping (biosimilars share MED_ABBR with reference products).</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>Discrepancy: The spec mentions permissible substitutions in the Additional Notes column but does not provide a complete structured list. Protocol Section 5.1.1 explicitly lists four substitution categories. The embedded code only has BORT&lt;-&gt;IXAZ and DARA self-sub; rituximab and biosimilar substitutions rely on the codelist mapping multiple codes to the same MED_ABBR. The spec should enumerate all substitution pairs.</t>
@@ -2832,8 +3348,6 @@
           <t>Spec=Y: Figure accurately represents the LOT1 BASE structure. Protocol=Y: 60-day window matches Section 5.1.1. Code=Y: All depicted concepts are implemented.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -2976,7 +3490,6 @@
           <t>Spec: N - uses simple min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP which is not yet defined; also garbled label text ('The end date for the 1date'). Protocol: Y - defines LOT1 end as earliest qualifying event with clear priority. Code: Y - implements priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCON &gt; CENSORED) which correctly reflects protocol priority; maintenance not yet integrated but logged as pending (line 4037).</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>Original spec uses min() of 5 dates including LOT1_BASE_MAINT_END_DT_TEMP, but the code uses a priority-based CASE statement (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED) rather than a simple minimum. The spec's label is garbled ('The end date for the 1date' should read 'The end date for the base period'). The inclusion of LOT1_BASE_MAINT_END_DT_TEMP in the min() is not applicable as maintenance is not enabled and is intentionally out of scope (confirmed by code comment at lot_program.R line 4037-4038).</t>
@@ -3029,7 +3542,6 @@
           <t>Spec: N - defines LOT1_END_DT_ORIG as a distinct variable for multi-step processing. Protocol: Y - protocol defines end date determination without specifying intermediate storage. Code: N - code does not create a separate LOT1_END_DT_ORIG variable; it computes the final end date directly in one step. The spec's multi-step approach (TEMP -&gt; ORIG -&gt; extend) differs from the code's single-pass approach.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_DT_ORIG as '= LOT1_END_DT_TEMP' (a copy). The code does not implement this intermediate variable. Instead, the code computes LOT1_BASE_END_DT directly using a priority-based CASE statement at lot_program.R lines 4018-4028. The multi-step approach in the spec (calculate TEMP, save ORIG, then extend) is an implementation design choice that the code handles differently.</t>
@@ -3082,7 +3594,6 @@
           <t>Spec: N - uses numeric codes 1-7 with date-matching logic and includes DEATH (4) as a separate end reason distinct from CENSOR. Protocol: Y - defines end reasons consistent with code priority (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). Code: Y - uses string end reasons ('SCT_AUTO', 'SCT_ALLO', 'SCT_CART', 'MED_ADD', 'DISCONTINUATION', 'CENSORED') with priority-based CASE; death is subsumed into CENSORED via OBS_END_DT.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>Multiple discrepancies: (1) Spec uses numeric codes (1-7) while code uses descriptive strings ('DISCONTINUATION', 'MED_ADD', 'CENSORED', 'SCT_AUTO', 'SCT_ALLO', 'SCT_CART'). (2) Spec has DEATH as a separate end reason (code 4); code subsumes death into CENSORED since DEATH_DT is incorporated into OBS_END_DT/ENDDATE. (3) Spec determines end reason by matching LOT1_END_DT_TEMP against each candidate date; code uses explicit priority-based CASE (SCT &gt; MED_ADD &gt; DISCONTINUATION &gt; CENSORED). (4) Spec's if/else chain checks LOT1_END_DT_TEMP against LOT1_DISCON_DT first, giving DISCONTINUATION highest priority among non-SCT reasons; code gives MED_ADD higher priority than DISCONTINUATION (when MED_ADD &lt;= DISCON). (5) Spec includes LOT1_BASE_MAINT_END_DT_TEMP in the initial min() which could set end reason to 2 (NEW MED) - maintenance is not yet implemented.</t>
@@ -3135,7 +3646,6 @@
           <t>Spec: N - defines LOT1_EXTEND_FLG as explicit 60-day extension from discontinuation. Protocol: N - protocol describes extending LOT1 for HSCT during conditioning but the code implements this differently. Code: Y - handles HSCT-during-conditioning via SCT priority in end reason CASE statement rather than a separate extension flag. The clinical intent is preserved but the implementation architecture differs significantly.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_FLG as a multi-step process: (1) check if LOT1 ended due to discontinuation, (2) check if HSCT occurred within 60 days, (3) extend LOT1 end date to include HSCT. The code does NOT implement this variable. Instead, the code gives SCT events highest priority in the LOT1_BASE_END_REASON CASE statement (lot_program.R lines 4001-4011), so if an SCT event occurs before discontinuation, it directly sets the end reason to SCT_AUTO/SCT_ALLO/SCT_CART. The 60-day extension concept from the spec is architecturally different from the code's priority-based approach. The code also logs that maintenance integration is pending (line 4037-4038).</t>
@@ -3188,7 +3698,6 @@
           <t>Spec: N - defines variable as LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. Protocol: N - does not explicitly name this metric. Code: Y - does not implement this variable (the code's architecture does not require it since SCT priority replaces the extension concept).</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>Spec defines LOT1_EXTEND_LENGTH = LOT1_END_DT_TEMP - LOT1_END_DT_ORIG. This variable is not implemented in the R code because the code does not use the multi-step extension approach. The code's priority-based CASE statement makes this variable unnecessary in the current implementation.</t>
@@ -3241,7 +3750,6 @@
           <t>Spec: N - defines a multi-step update process for end reason. Protocol: N - does not define a 'switch' concept explicitly. Code: Y - computes final end reason in single CASE statement without intermediate switch step.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>Spec defines LOT1_END_REASON_SWITCH as an updated version of LOT1_END_REASON_TEMP after HSCT extension logic. The code does not implement this as a separate variable. The code's single-pass LOT1_BASE_END_REASON (lot_program.R lines 4001-4017) serves as the final end reason. The spec's multi-step approach (TEMP -&gt; extend -&gt; SWITCH) is collapsed into one computation in the code.</t>
@@ -3294,7 +3802,6 @@
           <t>Spec: N - defines SWITCH_FLG based on LOT1_SAME_CLASS_1ST_DT which is not found in the code. Protocol: N - references same-class switching conceptually but does not define a specific flag variable. Code: Y - does not implement SWITCH_FLG; handles same-class via permissible_subs (lines 3346-3354) which treats certain within-class switches as part of the same LOT.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>Spec defines SWITCH_FLG = 1 if LOT1_SAME_CLASS_1ST_DT &lt;= LOT1_END_DT_TEMP. Neither LOT1_SAME_CLASS_1ST_DT nor SWITCH_FLG are implemented in the R code. The code handles same-class medication changes through the permissible substitutions mechanism (lot_program.R lines 3346-3354) rather than a separate flag. The spec's SWITCH_FLG concept is not present in the current codebase.</t>
@@ -3347,7 +3854,6 @@
           <t>Spec: N - includes additional logic to reset flag to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (HSCT occurred after LOT1 ended). Protocol: Y - defines single AUTO HSCT criteria. Code: Y - computes flag based on AUTO dates and tandem validation but does not reset to 0 based on LOT1_END_DT_TEMP; instead, the SCT priority logic in Step S16 handles this implicitly.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>Spec includes logic to set LOT1_HSCT_AUTO_SING_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1 (i.e., the HSCT occurred after the LOT ended). The code at lot_program.R lines 3911-3917 does not include this temporal filter - the flag is set purely based on AUTO date existence and tandem validation. However, in the code's Step S16 end reason logic (lines 4001-4011), SCT events are only used if LOT1_TX_ENDDATE &lt;= other end dates, effectively achieving the same clinical filtering.</t>
@@ -3400,7 +3906,6 @@
           <t>Spec: N - includes reset logic if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. Protocol: Y - defines tandem as 2 AUTO within 180 days with no ALLO between. Code: Y - implements tandem flag matching protocol definition; temporal filtering handled implicitly by Step S16 priority logic.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>Spec includes logic to reset LOT1_HSCT_AUTO_TAND_FLG to 0 if LOT1_END_DT_TEMP &lt; LOT1_TX_AUTO_DT_1. The code (lot_program.R lines 3904-3909) does not include this reset. Similar to SING_FLG, the temporal relationship is handled by Step S16's SCT priority logic rather than modifying the flag itself.</t>
@@ -3453,7 +3958,6 @@
           <t>Spec: N - defines explicit LOT1_TX_AUTO_MAX_DT variable. Protocol: Y - defines which AUTO date is the latest valid one. Code: Y - has equivalent data (AUTO_DT_1, AUTO_DT_2) but does not create a named LOT1_TX_AUTO_MAX_DT variable.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_MAX_DT as a named variable. The code does not create this specific variable but has the underlying data (AUTO_DT_1, AUTO_DT_2 at lot_program.R lines 3901-3902). The max valid AUTO date can be derived from the existing variables.</t>
@@ -3506,7 +4010,6 @@
           <t>Spec: N - defines explicit combined flag. Protocol: Y - concept is clear. Code: Y - does not create combined flag but has constituent flags (TAND and SING) from which it can be derived.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>Spec defines LOT1_TX_AUTO_FLG as a combined flag. The code does not create this specific variable but has LOT1_SCT_AUTO_TAND_FLG and LOT1_SCT_AUTO_SING_FLG (lot_program.R lines 3904-3917) from which the combined flag is trivially derivable.</t>
@@ -3559,7 +4062,6 @@
           <t>Spec: N - updates TEMP variable iteratively to HSCT date. Protocol: N - describes extending to include HSCT. Code: Y - uses LOT1_TX_ENDDATE (day before LOT-ending SCT) as the end date when SCT has priority. Key difference: spec extends LOT1 TO the HSCT date; code sets end to day BEFORE the LOT-ending SCT (which is the next AUTO after the included one).</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>Spec updates LOT1_END_DT_TEMP to the included HSCT date (AUTO_DT_1 for single, AUTO_DT_2 for tandem). The code's LOT1_TX_ENDDATE is date_sub(ENDING_AUTO_DT, 1) where ENDING_AUTO_DT is the NEXT AUTO beyond what's included (AUTO_DT_2 for single, AUTO_DT_3 for tandem). This means the code's end date is the day before the LOT-ending SCT, not the date of the included SCT. The architectural approach differs significantly between spec and code.</t>
@@ -3612,7 +4114,6 @@
           <t>Spec: Y - defines LOT1_BASE_MEDS as induction medications from LOT1_BASE dataset. Protocol: Y - defines induction regimen as medications in the induction window. Code: Y - implements via concat_ws/sort_array/collect_set of MED_ABBR from lot1_induction_meds.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -3665,7 +4166,6 @@
           <t>Spec: N - defines LOT1_BASEMAINT_START with specific logic but maintenance is not enabled. Protocol: - (maintenance concept defined in protocol but not currently in scope for implementation). Code: N - maintenance intentionally not enabled; explicitly logged at line 4037-4038. This is a deliberate scope decision, not an implementation gap.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_START with detailed conditions (120-day gap check, comparison with other end events). Maintenance is NOT ENABLED in the current implementation. The code explicitly logs that maintenance specs are not yet provided (lot_program.R lines 4037-4038). This is a deliberate scope decision - maintenance variables in the spec are aspirational and will require future implementation when maintenance is brought into scope.</t>
@@ -3718,7 +4218,6 @@
           <t>Spec: N - defines variable from LOT1_BASE_MAINT dataset but maintenance is not enabled. Protocol: - (defines maintenance medication concept but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_TYP from the LOT1_BASE_MAINT input dataset. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable that will require future implementation when maintenance is brought into scope.</t>
@@ -3771,7 +4270,6 @@
           <t>Spec: N - defines complex maintenance end date logic but maintenance is not enabled. Protocol: - (describes maintenance end conceptually but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END with detailed conditional logic. MAINTENANCE IS NOT ENABLED in the current implementation. This is an aspirational spec variable pending future scope decision.</t>
@@ -3824,7 +4322,6 @@
           <t>Spec: N - defines maintenance medication flags but maintenance is not enabled. Protocol: - (defines maintenance medications conceptually but not in scope). Code: N - maintenance intentionally not enabled. Induction med flags exist separately.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_MED_[MED] for BORT, DARA, IXAZ, LENA, CARF. MAINTENANCE IS NOT ENABLED in the current implementation. Induction medication flags (LOT1_MED_BORT, etc.) are implemented at lot_program.R Step S10 lines 3389 but these are separate from the maintenance flags. Aspirational spec variable pending future scope decision.</t>
@@ -3877,7 +4374,6 @@
           <t>Spec: N - defines maintenance end reason with numeric codes but maintenance is not enabled. Protocol: - (describes maintenance end conceptually but not in scope). Code: N - maintenance intentionally not enabled.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>Spec defines LOT1_BASEMAINT_END_REASON with numeric codes (1-6). MAINTENANCE IS NOT ENABLED in the current implementation. Additionally, the spec uses 6 values (1-6) while the base end reason has 7 (1-7, including CART) - the maintenance end reason omits CART (7), which may be intentional or an oversight. Aspirational spec variable pending future scope decision.</t>
@@ -3930,7 +4426,6 @@
           <t>Spec: - (not present). Protocol: - (defines end date concept but spec only has TEMP versions). Code: Y - implements LOT1_BASE_END_DT as the final computed end date. This variable is missing from the original spec which only has LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never creates the final non-temporary version.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_DT_TEMP and LOT1_END_DT_ORIG but never defines the final LOT1_BASE_END_DT. The code creates this as the definitive end date at lot_program.R Step S16 lines 4018-4028. The spec should include this final variable to show the output of the LOT1_BASE_END section.</t>
@@ -3983,7 +4478,6 @@
           <t>Spec: - (not present as final variable; only TEMP and SWITCH versions). Protocol: - (defines end reasons conceptually). Code: Y - implements LOT1_BASE_END_REASON as the final string-valued end reason.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The spec defines LOT1_END_REASON_TEMP and LOT1_END_REASON_SWITCH with numeric codes (1-7) but never creates the final LOT1_BASE_END_REASON. The code creates this with string values at lot_program.R Step S16 lines 4001-4017.</t>
@@ -4036,7 +4530,6 @@
           <t>Spec: - (not present). Protocol: - (concept exists via 60-day SCT window rule). Code: Y - implemented at Step S15 lines 3963-3972 and carried through to lot1_base_end.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code computes LOT1_1ST_SCT_DT at lot_program.R Step S15 (lines 3963-3972) as the earliest SCT of any type. This is useful for validating the protocol's 60-day window rule (SCT must occur within 60 days of induction/maintenance end to be continuation of LOT). The spec should include this variable.</t>
@@ -4089,7 +4582,6 @@
           <t>Spec: - (not present as standalone variable; referenced indirectly via SCT_ALLO end reason). Protocol: - (defines ALLO as always ending LOT). Code: Y - implemented at Step S15 line 3929 and used in end date/reason calculations.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_ALLO_DT at lot_program.R Step S15 (line 3929) and uses it in the LOT1_TX_ENDDATE and LOT1_TX_ENDDATE_REASON calculations. The protocol explicitly states that any ALLO SCT ends the current LOT (Section 5.1.1). The spec references SCT_ALLO as end reason code 6 but does not define FIRST_ALLO_DT as a standalone variable.</t>
@@ -4142,7 +4634,6 @@
           <t>Spec: - (not present as standalone variable; referenced indirectly via CART end reason code 7). Protocol: - (defines CAR-T as starting new LOT with 30-day consolidation rule). Code: Y - implemented at Step S15 line 3930.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>Variable missing from original spec. The code tracks FIRST_CART_DT at lot_program.R Step S15 (line 3930). The protocol defines CAR-T as always starting a new LOT (Section 5.1.2) with a 30-day supportive agent consolidation rule. The spec has CART as end reason code 7 but does not define FIRST_CART_DT as a standalone variable.</t>
@@ -4195,7 +4686,6 @@
           <t>Spec: - (not defined as a parameter; implicitly used but not documented). Protocol: - (defines discontinuation concept but does not specify exact gap threshold). Code: Y - implements as configurable parameter defaulting to 90 days at line 73, applied at line 3376.</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>Parameter missing from original spec. The code uses lot_discon_gap_days=90 (lot_program.R line 73) to determine whether a patient is truly discontinued vs censored. This critical threshold affects whether LOT1_BASE_DISCON_DT is set or left NULL. The spec should document this parameter as it directly affects the LOT1_END_REASON classification.</t>
@@ -4248,7 +4738,6 @@
           <t>Spec: - (not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1 under MAP algorithm). Code: Y - implemented as configurable parameter defaulting to 28 days at line 74.</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
       <c r="K26" t="inlineStr">
         <is>
           <t>Parameter missing from original spec's LOT1_BASE_END tab. The code uses medical_day_supply=28 (lot_program.R line 74) for MAP_END_DT calculation on medical claims. While this is defined in the MAP section (5B), it directly affects LOT1_BASE_DISCON_DT and should be cross-referenced here. Protocol Section 5.1.1 explicitly states the 28-day assumption.</t>
@@ -4301,7 +4790,6 @@
           <t>Spec: - (not defined in LOT1_BASE_END tab). Protocol: - (duration concept implied). Code: Y - computed at Step S10 lines 3447-3455 with priority MED_ADD &gt; DISCON &gt; CENSORED.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
       <c r="K27" t="inlineStr">
         <is>
           <t>Variable missing from original spec's LOT1_BASE_END tab. The code computes LOT1_BASE_LENGTH at lot_program.R Step S10 (lines 3447-3455) using a priority-based CASE matching the same hierarchy as LOT1_BASE_END_DT. Note: this is computed in the LOT1_BASE step (S10) rather than LOT1_BASE_END (S16), but it represents the base period duration which should be documented here.</t>
@@ -4354,7 +4842,6 @@
           <t>Spec: - (not defined). Protocol: - (defined in Section 5.1.1). Code: N - not applicable because maintenance is not enabled. This protocol rule will only be relevant when maintenance is brought into scope.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr">
         <is>
           <t>Protocol rule not in spec or code. Protocol Section 5.1.1 states that if SCT is not followed by maintenance within 180 days, the LOT ends at the SCT date. NOT APPLICABLE in current implementation because maintenance is not enabled. This rule should be implemented if/when maintenance is brought into scope.</t>
@@ -4407,7 +4894,6 @@
           <t>Spec: - (permissible substitutions not documented in LOT1_BASE_END tab). Protocol: - (defined in Section 5.1.1). Code: Y - implemented via permissible_subs table joined into base_meds CTE at Step S10 lines 3346-3354.</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr">
         <is>
           <t>Concept missing from original spec's LOT1_BASE_END tab. The code implements permissible substitutions by expanding base_meds to include substitutes (lot_program.R Step S10 lines 3346-3354). This is critical for correct LOT1_BASE_1ST_ADD_MED_DT calculation: without it, a permissible substitute (e.g., daratumumab/hyaluronidase replacing daratumumab) would incorrectly trigger a MED_ADD end reason. Protocol Section 5.1.1 explicitly defines which substitutions are permissible.</t>
@@ -4460,7 +4946,6 @@
           <t>Spec: - (not documented). Protocol: - (ambiguous on steroid role in discontinuation). Code: Y - steroids included in discontinuation with explicit code comment noting this is a design decision (lines 3355-3359) that stakeholders may want to change.</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
           <t>Design decision missing from original spec. The code includes steroids in the LOT1_BASE_DISCON_DT calculation (lot_program.R Step S10 lines 3355-3359) but documents this as a deliberate choice with a note for stakeholder review. The spec should document whether steroids should extend the discontinuation date, as this directly affects LOT1_BASE_END_DT for patients whose last active medication is a steroid.</t>
@@ -4603,8 +5088,6 @@
           <t>Spec: Y - correctly describes min(DATE_SERVICE) logic for first and subsequent MAPs. Protocol: Y - aligns with treatment episode start definitions. Code: Y - aggregate() state machine correctly initializes MAP_START_DT on first claim (CASE 1) and on new MAP boundary (CASE 2).</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4657,8 +5140,6 @@
           <t>Spec: Y - describes pushout=0 for first claim, pushout logic for subsequent, reset after rx gap, and stop when beyond both runouts. Protocol: Y - aligns with medication availability period definitions. Code: Y - aggregate() state machine implements all four pharmacy scenarios correctly per Figure 3.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4711,8 +5192,6 @@
           <t>Spec: Y - correctly describes medical runout as DATE_SERVICE + DAY_SUPPLY - 1 with no pushout. Protocol: Y - medical runout = date of medical claim + 28 days. Code: Y - implements greatest(existing, new) with no pushout; DAY_SUPPLY=28 for medical.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4765,8 +5244,6 @@
           <t>Spec: Y - correctly describes max of pharmacy and medical runout dates. Protocol: Y - MAP end determined by when medication availability ceases from both sources. Code: Y - greatest() of both runouts used in both CASE 2 (close MAP) and finalize function; QC validates this invariant.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4819,8 +5296,6 @@
           <t>Spec: Y - correctly defines sequential numbering starting at 1. Protocol: Y - treatment episodes numbered sequentially. Code: Y - accumulator starts at 0, CASE 1 sets to 1, CASE 2 increments by 1.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4873,8 +5348,6 @@
           <t>Spec: Y - correctly defines as =MED_ABBR. Protocol: Y - medication identification consistent. Code: Y - simple alias from MED_ABBR to MAP_MED_TYPE at line 3283.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4927,8 +5400,6 @@
           <t>Spec: Y - correctly defines as =MED_CLASS. Protocol: Y - therapeutic class assignment consistent. Code: Y - simple alias from MED_CLASS to MAP_MED_CLASS; min() used as deterministic tie-break.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -4981,8 +5452,6 @@
           <t>Spec: Y - correctly describes 90-day gap logic for both mid-sequence and last MAP cases. Protocol: Y - 90-day discontinuation threshold matches. Code: Y - lead() window function + datediff &gt;= 90 implements both cases; uses OBS_END_DT for last MAP.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5035,8 +5504,6 @@
           <t>Spec: Y - correctly describes stacking concept. Protocol: Y - all medication MAPs combined. Code: Y - implementation handles all medications in one pass via GROUP BY MED_ABBR, so map_stacked = map_med is correct. No separate per-medication datasets needed.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol. The spec describes creating individual MAP_[MED] datasets and then stacking; the R code achieves the same result in a single pass by grouping on MED_ABBR.</t>
@@ -5179,8 +5646,6 @@
           <t>Spec: Y - correctly states CODE is the code used to identify the medication. Protocol: Y - confirms NDC and HCPCS codes are the identification method for MM therapies. Code: Y - implements matching via codelist join with proper normalization.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol. Note: the code additionally checks BILL_PROC_CD and medical NDC fields beyond what the spec explicitly names, but this is consistent with the spec's intent to capture all relevant codes.</t>
@@ -5233,8 +5698,6 @@
           <t>Spec: Y - correctly lists NDC and HCPCS as code type values. Protocol: Y - confirms these are the two code type categories. Code: Y - uses CL_CODE_TYPE from codelist with values 'NDC' and 'HCPCS'.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5287,8 +5750,6 @@
           <t>Spec: Y - correctly identifies Medical and Pharmacy as claim types. Protocol: Y - confirms pharmacy and medical benefit claims are the two sources. Code: Y - hardcodes 'medical' for T_MEDICAL sources and 'pharmacy' for T_RX sources.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5341,8 +5802,6 @@
           <t>Spec: Y - correctly defines DAY_SUPPLY logic for pharmacy (from source) and medical (28), with filtering and dedup rules. Protocol: Y - confirms 28-day default for medical and missing/anomalous pharmacy claims. Code: Y - implements all rules: hardcoded 28 for medical via config, actual DAYS_SUP for pharmacy, filters pharmacy &lt; 1 or NULL, deduplicates via max(DAY_SUPPLY).</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol. The spec label says 'Days supply found on pharmacy claims' which is slightly misleading since medical claims also receive a DAY_SUPPLY value (28), but the definition section correctly explains both cases.</t>
@@ -5395,8 +5854,6 @@
           <t>Spec: Y - correctly defines DATE_SERVICE as the service date filtered between INDEX_DATE and ENDDATE inclusive, with proper dedup rules. Protocol: Y - confirms observation period bounds the claim window. Code: Y - implements FST_DT for medical, FILL_DT for pharmacy, filters to [INDEX_DATE, OBS_END_DT], and deduplicates by (PATID, MED_ABBR, DATE_SERVICE, CLAIM_TYPE). Note: spec uses 'ENDDATE' while code uses 'OBS_END_DT' - these represent the same concept (patient observation end date).</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol. Minor naming difference: spec references ENDDATE while code uses OBS_END_DT (both represent the patient's observation end date defined as earliest of death, disenrollment, or study end).</t>
@@ -5449,8 +5906,6 @@
           <t>Spec: Y - correctly defines MED_ABBR as CL_MED_ABBR from codelist where CODE = CL_CODE. Protocol: Y - confirms MM therapies are enumerated with specific names. Code: Y - derives MED_ABBR from codelist join and uses it as a grouping key in deduplication.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5503,8 +5958,6 @@
           <t>Spec: Y - correctly defines MED_CLASS as CL_MED_CLASS from codelist where CODE = CL_CODE. Protocol: Y - confirms therapeutic classification of MM therapies. Code: Y - derives MED_CLASS from codelist join and uses min() for deterministic dedup (functionally identical since class is constant per medication).</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5557,8 +6010,6 @@
           <t>Spec: Y - correctly defines MED_COND as Yes/No based on conditioning flag in Tab 40. Protocol: Y - confirms conditioning regimens are relevant for SCT-related treatment. Code: Y - implements conditioning flag from mma_rollup with robust parsing (handles 'YES', 'YES mainly...', '1', 0, NULL) and maps to 'Yes'/'No'.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5611,8 +6062,6 @@
           <t>Spec: Y - correctly defines MED_other_cancer as Yes/No based on 'Used for other cancers' flag in Tab 40. Protocol: Y - confirms relevance of other cancer indications for study exclusions and sensitivity analyses. Code: Y - implements USED_FOR_OTHER_CANCERS flag from mma_rollup with robust parsing and maps to 'Yes'/'No'.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -5665,8 +6114,6 @@
           <t>Spec: N - PATID is completely absent from the original program specification's Section A variable list despite being an output column in the mma_med_processed dataset. Protocol: Y - patient-level identification is fundamental to the study design. Code: Y - PATID is a key column in every CTE and the final output, and is part of the dedup GROUP BY key.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>PATID is missing from the original spec's Section A: Defining Analytic Variables. The mma_med_processed output has exactly 10 columns, and PATID is one of them. It is present in the code as the first column of every CTE (lines 2939, 2959, 2979, 3007, 3049, 3072) and is part of the GROUP BY deduplication key (line 3084). The spec should include PATID as a defined variable.</t>
@@ -5719,8 +6166,6 @@
           <t>Spec: N - The original spec does not explicitly state the therapy scope limitation or the corticosteroid exclusion rule. It references Tab 40/41 for code lists but does not articulate the principle that only FDA-approved/NCCN MM oncology therapies are included, or that corticosteroids alone are excluded. Protocol: Y - explicitly states therapy universe and corticosteroid exclusion. Code: Y - implements via INNER JOIN to codelist which inherently restricts to listed codes only.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>The original spec does not include an explicit processing rule or note stating that: (1) only FDA-approved MM oncology therapies per NCCN guidelines are captured, and (2) receipt of corticosteroids alone does not constitute evidence of MM therapy. The protocol makes both points explicitly (Section 4.2 Inclusion Criterion 5 and Section 5). While the codelist in Tab 40/41 implicitly enforces this by not including standalone corticosteroid codes, the spec should document this as a stated rule.</t>
@@ -5773,8 +6218,6 @@
           <t>Spec: N - Not mentioned in the MMA_MED section despite being defined in the same Tab 40 reference data as MED_COND and MED_other_cancer. Protocol: Y - Extensively defines valid mono-maintenance therapies with specific NCCN guideline references. Code: N - The field exists in mma_rollup but is intentionally NOT carried into mma_med_processed; it is used in a downstream step (MONOMAINT_MED). Whether it should be added to mma_med_processed for completeness is a design decision.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>The original spec's MMA_MED section does not mention the MONOMAINTENANCE flag despite it being sourced from the same Tab 40 reference table as MED_COND and MED_other_cancer. The protocol extensively defines valid mono-maintenance therapies (Protocol Section 5.1, page 8). The R code defines it in mma_rollup (line 2763-2765) but does not carry it into mma_med_processed - it is used in a separate downstream step (MONOMAINT_MED, Tab 8). The spec should at minimum reference this flag's existence in Tab 40 even if it is processed in a later step.</t>
@@ -5827,8 +6270,6 @@
           <t>Spec: N - Not mentioned in the MMA_MED section despite being defined in the same Tab 40 reference data. Protocol: Y - Explicitly lists valid dual-maintenance therapy combinations with NCCN references. Code: N - The field exists in mma_rollup (line 2766-2771) but is intentionally NOT carried into mma_med_processed; it is used in a downstream step (DUALMAINT_MED). Whether it should be added to mma_med_processed is a design decision.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>The original spec's MMA_MED section does not mention the DUALMAINTENANCEWITH flag despite it being sourced from the same Tab 40 reference table as MED_COND and MED_other_cancer. The protocol defines 3 valid dual-maintenance combinations (Protocol Section 5.1, page 8): bortezomib/lenalidomide, carfilzomib/lenalidomide, daratumumab/lenalidomide. The R code defines it in mma_rollup (line 2766-2771) but does not carry it into mma_med_processed - it is used in a separate downstream step (DUALMAINT_MED, Tab 9). The spec should at minimum reference this field's existence in Tab 40.</t>
@@ -5881,8 +6322,6 @@
           <t>Spec: N - The original spec does not mention mesna or its exclusion. It relies entirely on the codelist to define the therapy universe without documenting specific exclusions. Protocol: Y - Explicitly names mesna as an excluded therapy with rationale. Code: Y - Implicitly excludes mesna by not including it in the codelist; INNER JOIN ensures non-listed codes are dropped.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>The original spec does not document the mesna exclusion. The protocol explicitly states in Section 5.1.2 (page 9) that mesna is excluded from LOTs. While the codelist implicitly enforces this exclusion, the spec should document it as a stated rule for transparency and auditability.</t>
@@ -5935,8 +6374,6 @@
           <t>Spec: N - The spec says to DELETE pharmacy claims with DAY_SUPPLY &lt; 1 or missing, which contradicts the protocol. Protocol: N - The protocol says to DEFAULT to 28 days, but this is what the protocol actually requires (marked N here because the current implementation does not match it). Code: Y - The code correctly implements what the SPEC says (delete), but the spec itself contradicts the protocol. Note: This is a case where the spec and code agree with each other (both say delete) but BOTH disagree with the protocol (which says default to 28).</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>MATERIAL DISCREPANCY: The protocol (Section 5.1.2, page 9) states 'When pharmacy claims are missing days supply, or when days supply values are anomalous, 28 days will be assumed.' However, the original spec instructs: 'If CLAIM_TYPE_SOURCE = pharmacy and (DAY_SUPPLY_SOURCE &lt; 1 or DAY_SUPPLY_SOURCE is missing) then delete.' The code implements the spec's delete behavior (lot_program.R line 3066). This means pharmacy claims with anomalous DAY_SUPPLY are lost rather than being preserved with a 28-day default. This could affect medication exposure calculations and LOT duration. The spec and code should be updated to default to 28 instead of deleting, per protocol.</t>
@@ -5989,8 +6426,6 @@
           <t>Spec: N - The original spec does not mention permissible substitutions or biosimilar equivalence. Protocol: N - The protocol defines these rules for LOT advancement (not directly for MMA_MED), so marking N as the MMA_MED section does not reflect them. Code: Y - The code handles substitutions downstream via permissible_substitutions table (lot_program.R line 3225 in MAP_MED step), not at the MMA_MED level. Whether equivalence should be defined at MMA_MED or downstream is a design decision.</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>The original spec does not document the protocol's permissible substitution rules (Protocol Section 5.1.2, page 9). These rules define which medication switches do NOT advance a LOT: rituximab/hyaluronidase equivalence, daratumumab/hyaluronidase equivalence, biosimilar/reference product equivalence, and bortezomib-to-ixazomib maintenance transition. While primarily a downstream LOT rule, the codelist design (Tab 40/41) must ensure consistent MED_ABBR mapping for equivalent products. The code handles this in MAP_MED via permissible_substitutions (line 3225), not in MMA_MED.</t>
@@ -6136,8 +6571,6 @@
           <t>Spec, protocol, and code all agree. Spec correctly defines the variable as the first AUTO SCT date within LOT1_START_DT to ENDDATE. Code adds the additional constraint of excluding AUTO events after the first ALLO/CART, which is consistent with protocol rule that ALLO/CART immediately end LOT1.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6190,8 +6623,6 @@
           <t>All sources agree. The second AUTO date is the next processed AUTO event after the first, within LOT1 boundaries.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6244,8 +6675,6 @@
           <t>Spec says '(LOT1_TX_AUTO_DT_2 - LOT1_TX_AUTO_DT_1 + 1) &lt;= 180' which matches code's 'datediff + 1 &lt;= 180'. However, the spec does NOT mention the &gt;=60 day minimum gap between tandem SCTs that the protocol explicitly requires ('&gt;=60 to &lt;=180 days apart'). The code enforces the 60-day gap via the AUTO date processing in Step S13 (sct_auto_gap_days=60), so protocol and code agree but spec omits the &gt;=60 day lower bound.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>Partial discrepancy: Spec omits the &gt;=60 day minimum gap between tandem AUTO SCTs. Protocol Section 5 clearly states 'at least two autologous SCTs &gt;=60 to &lt;=180 days apart.' The 60-day gap is enforced in code (Step S13 sct_auto_gap_days=60) but not explicitly stated in the spec's tandem flag definition.</t>
@@ -6298,8 +6727,6 @@
           <t>All sources agree. Single flag = has AUTO_DT_1 but not a valid tandem.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6352,8 +6779,6 @@
           <t>All three sources agree on the logic. Spec describes the iterative approach (iterate over ALLO SCTs, CAR-Ts); code implements the same via CTEs for earliest_non_auto, first_allo, first_cart, and ENDING_AUTO_DT. The spec's iteration description is more verbose but logically equivalent to the code's min/least approach.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6406,8 +6831,6 @@
           <t>All three sources agree on the reason coding (1=AUTO, 2=ALLO, 3=CART) and the logic to select the earliest event.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6460,8 +6883,6 @@
           <t>Spec definition says 'Set to min(LOT1_TX_AUTO_DT_1, LOT1_TX_ENDDATE)' which is incomplete. The code and protocol define it as the earliest of AUTO_DT_1, FIRST_ALLO_DT, and FIRST_CART_DT -- not LOT1_TX_ENDDATE. LOT1_TX_ENDDATE is a derived end date (day before the ending event), not the actual SCT date. Protocol and code agree on using actual first SCT dates.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>Discrepancy found: Spec defines LOT1_1ST_SCT_DT as 'min(LOT1_TX_AUTO_DT_1</t>
@@ -6529,8 +6950,6 @@
           <t>Spec, protocol, and code all agree on the core logic. The spec's pseudocode description of the 14-day windowing, 60-day gap, and 180-day tandem boundary adjustment matches the code's implementation. ALLO and CART use simple sequential ordering without windowing, as described in spec and implemented in code.</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6583,8 +7002,6 @@
           <t>Spec example matches code logic. The spec provides a detailed worked example (Patient A) that demonstrates the 14-day window, 60-day gap, and 180-day tandem boundary adjustment. Code implements this exactly with cfg parameters.</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6637,8 +7054,6 @@
           <t>Spec references Tab 47 and code implements both external codelist and embedded fallback codes. CPT 38241=AUTO and 38240=ALLO per AMA CPT definitions.</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6691,8 +7106,6 @@
           <t>All sources agree on end reason priority. Code explicitly checks that SCT end date occurs at or before medication addition and discontinuation dates before assigning SCT as the end reason.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6835,8 +7248,6 @@
           <t>Spec, protocol, and code all agree on INDEX_DATE definition. Spec mentions Tab 42 for MM dx codes. Protocol Section 4.2 Criterion 1 matches. Code implements strict (203.0x/C90.0x) for inpatient and broad (203.x/C90.x) for outpatient, with 30/60/90 day windows, consistent with protocol note about flagging 30/60 day pairs.</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6889,8 +7300,6 @@
           <t>All sources agree. Simple derivation from INDEX_DATE.</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6943,8 +7352,6 @@
           <t>All sources agree on age calculation method and &gt;=18 threshold.</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -6997,8 +7404,6 @@
           <t>All three sources agree on 6-month baseline, 30-day gap allowance, and binary flag logic.</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7051,8 +7456,6 @@
           <t>All sources agree. CE_f requires enrollment covering the index date with 30-day gap allowance.</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7105,8 +7508,6 @@
           <t>All sources agree on no-gap requirement and death-awareness for CE_3mosf. Code correctly uses member_enrollment (raw) rather than member_cont_enrollment to detect true gaps.</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7159,8 +7560,6 @@
           <t>All sources agree. Code correctly bounds follow-up therapy by death date to prevent post-death claims.</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7213,8 +7612,6 @@
           <t>All sources agree on baseline therapy exclusion logic. Code correctly excludes index_date from baseline period (baseline_end = index_date - 1).</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7267,8 +7664,6 @@
           <t>Spec: N - Definition column says 'any evidence of MM' but Additional Notes say 'non-diagnostic claim' - these contradict each other (flagged in QC review by Onkar Kshirsagar). Protocol: Y - Protocol discusses baseline MM evidence and smoldering identification. Code: Y - Code correctly implements non-diagnostic claim logic but defaults to disabled (apply_baseline_nondx_excl=FALSE).</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>Discrepancy found: The Definition column states 'Evidence of any MM' broadly while the Additional Notes specify 'non-diagnostic medical claim' specifically. The QC reviewer (Onkar Kshirsagar) flagged this inconsistency. The validated definition should specify 'non-diagnostic' per the Additional Notes and code implementation.</t>
@@ -7321,8 +7716,6 @@
           <t>Spec: N - Spec says only first of 2 codes must be in baseline, but QC reviewer noted both should be in baseline. Also protocol mentions inpatient (1 claim) vs outpatient (2 claims) distinction that spec omits. Protocol: Y - Protocol provides the authoritative definition with inpatient/outpatient distinction. Code: Y - Code implements 2 codes within 30 days with first_dt in baseline, matching the spec's stated rule (not the QC reviewer's correction).</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
         <is>
           <t>Discrepancy found: 1) Protocol specifies '&gt;=1 inpatient or &gt;=2 outpatient' distinction for other cancer that the spec omits. 2) QC reviewer (Onkar Kshirsagar) noted 'Both claims have to be in baseline' but the spec text says only the first of the 2 codes must be in the baseline period. Code follows the spec text (first_dt in baseline). The protocol also mentions 60/90 day flagging for consideration.</t>
@@ -7375,8 +7768,6 @@
           <t>Spec: N - Spec defines this as a separate variable but does not detail the follow-up period logic clearly. Protocol: N - Protocol mentions baseline exclusion for other cancer, not follow-up as separate criterion. Code: Y - Code only implements baseline other malignancy flag (OTHER_MALIGN_FLAG). No separate FU_other_malig flag exists in the code.</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
         <is>
           <t>Discrepancy found: The spec defines MM_FU_other as a separate variable for follow-up period other cancer evidence, but the code only implements OTHER_MALIGN_FLAG for the baseline period. The protocol's Exclusion Criterion 2 focuses on baseline period. If FU other cancer is needed, it would require a separate flag computation.</t>
@@ -7429,8 +7820,6 @@
           <t>All sources agree on pregnancy flag logic spanning baseline + follow-up. Code includes revenue code support per spec requirement.</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7483,8 +7872,6 @@
           <t>All sources agree. Code splits into baseline and follow-up clinical trial flags for granularity, which is consistent with protocol saying 'during the study period'.</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7537,8 +7924,6 @@
           <t>Spec: N - Spec mentions the July 15th rule for year-only death dates and Dec 31st rule when index &gt; July 15th, but does not mention the month-level edge case (when index_date &gt; 15th of death month, use month-end). Protocol: Y - Protocol says '15th of the month' without specifying the edge case, but the code correctly handles it. Code: Y - Code implements comprehensive logic including edge cases.</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
         <is>
           <t>Discrepancy found: The spec does not describe the month-level edge case where if index_date &gt; 15th of the death month, the death date is set to month-end instead of the 15th. This edge case is implemented in code (line 1996-1997) to prevent death_dt &lt; index_date. The protocol simply states '15th of the month' without addressing this edge case.</t>
@@ -7591,8 +7976,6 @@
           <t>All sources agree. ENDDATE = min(death, study_end), not including disenrollment.</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7645,8 +8028,6 @@
           <t>All sources agree. ENDDATE_CE = min(death, disenrollment, study_end).</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7699,8 +8080,6 @@
           <t>All sources agree on FU_DAYS computation.</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7753,8 +8132,6 @@
           <t>All sources agree on FU_DAYS_CE computation.</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7807,8 +8184,6 @@
           <t>All sources agree on the base cohort being all patients with &gt;=1 MM claim.</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7861,8 +8236,6 @@
           <t>Spec: N - Spec uses ICD-9-CM=203.0x for both inpatient and outpatient in the definition column, but the Additional Notes use 203.x (broader) for outpatient. Protocol: Y - Protocol says 'ICD-9-CM=203.0x or ICD-10-CM=C90.0x' for inpatient then '&gt;=2 medical claims for MM' for outpatient (broader). Code: Y - Code correctly uses strict codes (203.0x/C90.0x) for inpatient and broad codes (203.x/C90.x) for outpatient.</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
         <is>
           <t>Discrepancy found: The spec definition column uses ICD-9-CM=203.0x and ICD-10-CM=C90.0x for BOTH inpatient and outpatient claims, but the Additional Notes column uses broader codes 203.x and C90.x for outpatient. The protocol and code correctly distinguish strict (inpatient) from broad (outpatient) codes. The definition column should clarify this distinction.</t>
@@ -7915,8 +8288,6 @@
           <t>All sources agree on age &gt;=18 in index year.</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -7969,8 +8340,6 @@
           <t>All sources agree.</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8023,8 +8392,6 @@
           <t>All sources agree.</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8077,8 +8444,6 @@
           <t>All sources agree.</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8131,8 +8496,6 @@
           <t>All sources agree.</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8185,8 +8548,6 @@
           <t>Spec: N - Spec says 'non-diagnostic' codes but code does NOT require non-diagnostic claims for other cancer (per line 2314 comment: 'Attrition table does NOT require non-diagnostic claims for other cancer'). Protocol: Y - Protocol does not specify non-diagnostic for other cancer. Code: Y - Code correctly omits non-diagnostic requirement.</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>Discrepancy found: The spec mentions 'non-diagnostic diagnosis codes' for other cancer criterion, but neither the protocol nor the code requires non-diagnostic claims for other cancer identification. The code explicitly notes this (line 2314). The term 'non-diagnostic' appears to be erroneously carried over from the MM baseline diagnosis definition.</t>
@@ -8239,8 +8600,6 @@
           <t>All sources agree.</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8293,8 +8652,6 @@
           <t>All sources agree. Code correctly flags baseline and follow-up separately.</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8347,8 +8704,6 @@
           <t>All sources agree on final cohort construction with flexible IE criteria and exclusion defaults set to FALSE for criteria 7-9 as specified.</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>No discrepancy found. Aligned with protocol.</t>
@@ -8401,8 +8756,6 @@
           <t>Spec: N - The original spec does not define STUDY_PERIOD, study_start, study_end, id_start, or id_end as explicit variables. These critical date parameters are only implied by the DataPrep page. Protocol: Y - Protocol clearly defines study period (Jul 2015 - Jun 2025) and identification period (Jan 2016 - Jun 2025). Code: Y - Code parameterizes all four dates as cfg variables.</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr">
         <is>
           <t>Missing from spec: The StudyPop page does not explicitly define the study period (1 Jul 2015 - 30 Jun 2025) or identification period (1 Jan 2016 - 30 Jun 2025) as named variables. These critical parameters are defined in the DataPrep page but should be referenced or echoed in StudyPop for completeness.</t>
@@ -8455,8 +8808,6 @@
           <t>Spec: N - The spec defines CE_b referencing 'six months' but does not explicitly state the smoldering MM assumption or the clinical rationale for the baseline period. Protocol: Y - Protocol explains the smoldering assumption clearly. Code: Y - Code implements baseline_days=183 with explicit start/end dates.</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr">
         <is>
           <t>Missing from spec: The spec does not capture the protocol's key clinical rationale that untreated baseline patients are assumed to be smoldering MM until treatment in follow-up. This is important context for understanding why the baseline therapy exclusion exists (Protocol Section 4.2, Criterion 3).</t>
@@ -8509,8 +8860,6 @@
           <t>Spec: N - The spec mentions MM_FU_agents as 'FDA-approved MM oncology therapy' but does not explicitly state that corticosteroids alone do not qualify at the StudyPop level. Protocol: Y - Protocol is explicit about corticosteroid exclusion. Code: N - Code includes steroids in therapy codes for MM_FU_agents/MM_bl_agents flags; the steroid-only exclusion is deferred to LOT classification rather than being applied at the StudyPop inclusion/exclusion stage.</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr">
         <is>
           <t>Missing from spec: The spec does not explicitly state that corticosteroids alone do not count as evidence of MM therapy for MM_FU_agents or MM_bl_agents. The protocol is explicit (Section 4.2, Criterion 5). The code includes steroids in therapy event matching at the StudyPop level and defers the steroid-only exclusion to the LOT algorithm. This could cause patients on corticosteroids-only to be included/excluded incorrectly at the StudyPop stage.</t>
@@ -8563,8 +8912,6 @@
           <t>Spec: N - The spec describes individual criteria but does not capture the protocol's explicit statement about flexibility and the sole mandatory requirement. The spec's Section C partially addresses this but does not quote the mandatory requirement verbatim. Protocol: Y - Protocol is explicit. Code: Y - Code fully implements flexible criteria with interactive toggling and dynamic ordering.</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr">
         <is>
           <t>Missing from spec: The spec does not explicitly state the protocol's 'sole mandatory requirement' language or that all criteria beyond MM diagnosis and no-baseline-therapy are optional. This is critical context from Protocol Section 4.2 preamble that should be documented in the spec.</t>
@@ -8617,8 +8964,6 @@
           <t>Spec: N - The spec references Tab 42 for MM dx codes but does not explain the rationale for using broad codes or the insurance-vs-research context. Protocol: Y - Protocol explicitly states the rationale. Code: Y - Code implements both strict and broad code matching.</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr">
         <is>
           <t>Missing from spec: The spec references Tab 42 for MM codes but does not document the protocol's important note that all MM diagnosis codes should be considered because Optum CDM data is collected for insurance, not research purposes. This rationale (Protocol Section 4.2, Criterion 1 note) explains why broad codes (203.x/C90.x) are used for outpatient claims.</t>
@@ -8671,8 +9016,6 @@
           <t>Spec: N - Spec mentions 30-day window only; does not implement 60/90 day flagging or inpatient/outpatient distinction for other cancer. Protocol: N - Protocol specifies both 30-day window AND 60/90 day flagging AND inpatient/outpatient distinction, but these are partially implemented. Code: Y - Code implements 30-day window only; no 60/90 day other cancer flags; no inpatient/outpatient distinction.</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>Missing from spec: The spec does not include 60/90 day window flagging for other cancer or the inpatient (&gt;=1 claim) vs outpatient (&gt;=2 claims) distinction specified in Protocol Section 4.2 Exclusion Criterion 2. The code similarly only implements the 30-day window. Both spec and code should add other cancer flags for 60/90 day windows and distinguish inpatient from outpatient claims.</t>
@@ -8725,8 +9068,6 @@
           <t>Spec: N - The StudyPop page does not describe the data source or CDM characteristics. Protocol: Y - Protocol Section 4.4 provides comprehensive data source description. Code: Y - Code header documents CDM version and validates against data dictionary.</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>Missing from spec: The StudyPop page does not document the data source (Optum CDM). Protocol Section 4.4 provides important context: HIPAA-compliant, de-identified, ~15-20M lives/year, both medical and pharmacy benefits required, service dates from 2007. This should be referenced on the StudyPop page or a dedicated Data Source section.</t>
@@ -8779,11 +9120,2187 @@
           <t>Spec: N - The spec mentions death date generalization rules (15th of month, July 15th for year-only) but does not document the 6 death data sources or their ranking. Protocol: Y - Protocol Section 4.5 explicitly lists all sources. Code: Y - Code uses T_DOD.YMDOD which already reflects the CDM's source ranking.</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
         <is>
           <t>Missing from spec: The spec does not document the 6 ranked death data sources from Protocol Section 4.5. While the CDM pre-applies this ranking, documenting the sources is important for understanding data completeness and potential limitations (e.g., month-only vs year-only granularity depends on the source).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Definition (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Additional Notes (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Optum CDM Implementation</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>R Code Implementation</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status (OrigSpec/Protocol/Code)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Date Modified (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>QC Reviewed (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Discrepancy Found in Original Program Spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Classification</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>LOT2_PLUS_DEFINITION</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Second-line (LOT2) and later LOTs classification</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>Second-line (LOT2) and later LOTs: Indicated by initiation of new therapy or an SCT after the end of the previous LOT. The LOT rules described above apply to LOT2 and later LOTs with the caveat that for LOT2 and later LOTs the regimen identification window (to determine which MM treatments are present in the LOT) is 30 days instead of 60 days.</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.2: 'Second-line (L2) and later LOTs: Indicated by initiation of new therapy or an SCT after the end of the previous LOT (IL+/- maintenance or IL SCT + maintenance). The LOT rules described above apply to LOT2 and later LOTs with the caveat that for LOT2 and later LOTs the regimen identification window (to determine which MM treatments are present in the LOT) is 30 days instead of 60 days.'</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr"/>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Classification</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>MAX_LOT_COUNT</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Maximum number of LOTs per patient</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>Up to five lines of therapy will be identified for the entire follow-up period per patient.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'For each patient, up to five lines of therapy will be identified for the entire follow-up period.'</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Start</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_START_DT</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>LOT N start date (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>LOT N begins on the earlier of: (a) a SCT (allogeneic or an unplanned autologous SCT), CAR-T, or (b) the date of the first fill for an MM therapy following the end of the previous LOT.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 LOT start date: 'Subsequent LOTs will begin on the earlier of a SCT (allogeneic or an unplanned autologous SCT), CAR-T or the date of the first fill for an MM therapy following the end of the previous LOT.'</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Start</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_REGIMEN_WINDOW</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>LOT N regimen identification window (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>For LOT2-5: A LOT regimen includes all MM therapies received within 30 days on and following the start of the LOT.</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'A LOT regimen includes all MM therapies received within 60 (30) days on and following the start of LOT1 (LOT2-5).' (Madduri, 2021)</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Start</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MED_[MED]</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>[MED] is present in LOT N regimen (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>Binary flag (0/1). =1 if MAP_MED_TYPE=[MED] and LOTN_START_DT &lt;= MAP_START_DT &lt;= (LOTN_START_DT+29) then = 1. Else 0. Analogous to LOT1_MED_[MED] but with 30-day window.</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'For LOT1, the first therapy received is considered the induction therapy.' LOT2-5 use a 30-day window to identify the regimen (vs 60 days for LOT1).</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Start</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MED_CNT</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Count of distinct medications in LOT N regimen (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Count of distinct MM therapies present within the first 30 days of LOT N.</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Analogous to LOT1_MED_CNT using the 30-day regimen window for LOT2-5.</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr"/>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 End</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_END_DT</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>LOT N end date (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>The LOT will continue until the earliest of: (1) Substitution of a new MM treatment after the initial agent(s), (2) Discontinuation of all agents in the regimen, (3) Unplanned SCTs (autologous SCT &gt;180 days after previous autologous SCT in the LOT), (4) SCTs not followed by maintenance within 180 days, (5) Death, (6) Health plan disenrollment, (7) End of the study period, (8) End of maintenance regimen.</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 LOT end date: Defines 8 LOT end conditions. All rules from LOT1 apply identically to LOT2-5.</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr"/>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 End</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_END_REASON</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Reason LOT N ended (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Categorical: SUBSTITUTION / DISCONTINUATION / SCT_AUTO / SCT_ALLO / SCT_CART / DEATH / DISENROLLMENT / STUDY_END / MAINTENANCE_END. Same end reason definitions as LOT1.</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: Same end conditions and priority rules as LOT1.</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="inlineStr"/>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 End</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_BASE_LENGTH</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>LOT N base period duration in days (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Duration from LOTN_START_DT to LOTN_END_DT in days. Same calculation as LOT1_BASE_LENGTH.</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Data analysis: 'time between LOTs (mean, standard deviation, median, IQR, min, max) will be tabulated.'</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Permissible Substitutions</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_PERMISSIBLE_SUBS</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Permissible substitutions for LOT2-5</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>The following substitutions do not advance the LOT: (a) Substitution of the reference product for a biosimilar or vice versa, (b) Substitution of daratumumab for daratumumab/hyaluronidase and vice versa, (c) Substitution of rituximab for rituximab/hyaluronidase and vice versa, (d) Substitution of bortezomib induction therapy for ixazomib as a maintenance therapy.</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: These permissible substitutions apply to all LOTs (LOT1 through LOT5).</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 CAR-T</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_CART_FLG</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Flag: LOT N is a CAR-T LOT (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Binary flag (0/1). =1 if the LOT consists of a CAR-T cellular therapy infusion. CAR-T cellular therapy infusions should be classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.2: 'CAR-T: CAR-T cellular therapy infusions should be classified as their own LOT. Therapies (including supportive agents, e.g., corticosteroids) given within 30 days of CAR-T cellular therapy are consolidated as part of the CAR-T LOT.'</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 SCT</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_SCT_FLG</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>LOT-specific binary variable for SCT during LOT N (N=2-5)</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT. SCT is operationalized as &gt;= 1 non-diagnostic procedure code for an SCT. Same processing logic as LOT1 (14-day window, 60-day gap, tandem detection).</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1: 'Stem cell transplant (SCT): A LOT-specific binary variable is created to classify whether patients have an SCT during the LOT. SCT is operationalized as &gt;= 1 non-diagnostic procedure code for an SCT.'</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Allogeneic</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_ALLO_LOT</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Allogeneic SCT as own LOT</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Presence of an allogeneic SCT immediately ends a LOT and starts a new LOT. The new LOT will consist entirely of the allogeneic SCT and no other MM therapies.</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Allogeneic SCT: Presence of an allogeneic SCT immediately ends a LOT, and starts a new LOT. The new LOT will consist entirely of the allogeneic SCT and no other MM therapies.'</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr"/>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Time Between LOTs</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>TIME_BETWEEN_LOTS</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Time between consecutive LOTs</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Time in days from LOTN_END_DT to LOT(N+1)_START_DT. Distribution (mean, standard deviation, median, IQR, min, max) to be tabulated.</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Data analysis: 'The distribution of number of LOTs per patient and time between LOTs (mean, standard deviation, median, IQR, min, max) will be tabulated.'</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>LOT2-5 Distribution</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>NUM_LOTS</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Total number of LOTs per patient</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Integer (1-5). Count of sequential LOTs identified for the patient during follow-up.</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.3 Data analysis: 'The distribution of number of LOTs per patient and time between LOTs (mean, standard deviation, median, IQR, min, max) will be tabulated.'</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented in spec or code</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr"/>
+      <c r="L16" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for LOT2-5</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
+    <col width="33" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Variable Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Definition (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Additional Notes (Validated from Protocol)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Optum CDM Implementation</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>R Code Implementation</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status (OrigSpec/Protocol/Code)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Sync Status Notes</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Date Modified (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>QC Reviewed (Initials + Date)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Discrepancy Found in Original Program Spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Definition</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_REGIMEN_DEF</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance regimen definition</t>
+        </is>
+      </c>
+      <c r="D2" s="1" t="inlineStr">
+        <is>
+          <t>A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available (see valid maintenance therapies below). Maintenance is not required to be prescribed continuously for the duration of the 120 day period. Furthermore, the maintenance therapy must have been a part of the LOT's initial regimen (for LOT1 the initial regimen includes all MM therapies identified during the first 60 days of LOT1, for LOT2-5 the initial regimen is defined as all MM therapies identified during the first 30 days of the LOT).</t>
+        </is>
+      </c>
+      <c r="E2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 Maintenance regimen: 'A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available. Maintenance is not required to be prescribed continuously for the duration of the 120 day period. Furthermore, the maintenance therapy must have been a part of the LOT's initial regimen.'</t>
+        </is>
+      </c>
+      <c r="F2" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G2" s="1" t="inlineStr">
+        <is>
+          <t>lot_program.R lines 4037-4038 note maintenance specs not yet provided</t>
+        </is>
+      </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>NNP</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>Protocol defined; lot1baseend has placeholder maintenance vars (LOT1_BASEMAINT_*) but full logic not implemented</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr"/>
+      <c r="K2" s="1" t="inlineStr"/>
+      <c r="L2" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Definition</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_MIN_PERIOD</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Minimum maintenance period (non-SCT)</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t>120 days. A valid maintenance regimen requires a period of 120 days or longer during which only a valid maintenance therapy is available.</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'A maintenance regimen is a period of 120 days or longer during which only a valid maintenance therapy is available.'</t>
+        </is>
+      </c>
+      <c r="F3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G3" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr"/>
+      <c r="K3" s="1" t="inlineStr"/>
+      <c r="L3" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Definition</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_POST_SCT_MIN_PERIOD</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Minimum maintenance period after SCT</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>30 days (minimum). Following an autologous SCT (within 180 days of the HSCT or in the case of a tandem autologous HSCT within 180 days of the second HSCT). The expectation after an HSCT is for a maintenance period and thus instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period.</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Following an autologous SCT... instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period. Any valid maintenance regimens present after a single autologous SCT or after the second SCT of a tandem autologous SCT will be considered. These maintenance drugs must have been part of the LOT's initial regimen.'</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr"/>
+      <c r="K4" s="1" t="inlineStr"/>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Definition</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_POST_SCT_FU_EXCEPTION</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance period shortened by end of follow-up after SCT</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>If a full 30-day period is unable to be observed due to the end of follow-up, whatever days are available will be the maintenance period to avoid a new LOT starting immediately before the end of follow-up.</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'If a full 30-day period is unable to be observed due to the end of follow-up, we will still count whatever days are available as a maintenance period to avoid a new LOT starting immediately before the end of follow-up.' Also footnote 1: 'If an otherwise valid maintenance period that came after an SCT did not reach 120 days due to follow-up ending, then that period is still assigned as maintenance.'</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr"/>
+      <c r="K5" s="1" t="inlineStr"/>
+      <c r="L5" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Situation 1</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_TRANSITION_RULE</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>LOT regimen transitions into maintenance</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>A maintenance regimen may occur when the LOT's initial regimen transitions into a maintenance regimen, such that non-maintenance medications present during the initial regimen are discontinued leaving only maintenance medications. For example, a patient has an initial regimen of cyclophosphamide and daratumumab, and then discontinues cyclophosphamide leaving only daratumumab, which is a valid mono maintenance.</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 Maintenance regimen situation 1: 'The LOT's initial regimen transitions into a maintenance regimen, such that non-maintenance medications present during the initial regimen are discontinued leaving only maintenance medications.'</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr"/>
+      <c r="K6" s="1" t="inlineStr"/>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Situation 2</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_POST_SCT_RULE</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance following autologous SCT</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="inlineStr">
+        <is>
+          <t>Following an autologous SCT (within 180 days of the HSCT or in the case of a tandem autologous HSCT within 180 days of the second HSCT). Any valid maintenance regimens present after a single autologous SCT or after the second SCT of a tandem autologous SCT will be considered. These maintenance drugs must have been part of the LOT's initial regimen.</t>
+        </is>
+      </c>
+      <c r="E7" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1 Maintenance regimen situation 2: 'Following an autologous SCT (within 180 days of the HSCT...). The expectation after an HSCT is for a maintenance period and thus instead of the usual 120 days, we check for a valid 30-day (minimum) maintenance period.'</t>
+        </is>
+      </c>
+      <c r="F7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G7" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr"/>
+      <c r="K7" s="1" t="inlineStr"/>
+      <c r="L7" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Valid Mono Maintenance</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_LENA_MONO</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Lenalidomide monotherapy</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>Lenalidomide monotherapy. NCCN Preferred Regimen for both transplant and non-transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Lenalidomide monotherapy (NCCN Preferred Regimen for both transplant and non-transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr"/>
+      <c r="K8" s="1" t="inlineStr"/>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Valid Mono Maintenance</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_BORT_MONO</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>Bortezomib monotherapy</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>Bortezomib monotherapy. NCCN Other Recommended Regimen for both transplant and non-transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Bortezomib monotherapy (NCCN Other Recommended Regimen for both transplant and non-transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr"/>
+      <c r="K9" s="1" t="inlineStr"/>
+      <c r="L9" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Valid Mono Maintenance</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_DARA_MONO</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>Daratumumab monotherapy</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>Daratumumab monotherapy. NCCN Other Recommended Regimen for transplant candidates. Protocol notes: any maintenance medications listed will be considered for all patients regardless of transplant status.</t>
+        </is>
+      </c>
+      <c r="E10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Daratumumab monotherapy (NCCN Other Recommended Regimen for transplant candidates)'. 'Any of the maintenance medications listed above will be considered maintenance medications for all patients, regardless of transplant status.'</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G10" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Valid Mono Maintenance</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_IXAZ_MONO</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Ixazomib monotherapy</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Ixazomib monotherapy. NCCN Other Recommended Regimen for both transplant and non-transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Ixazomib monotherapy (NCCN Other Recommended Regimen for both transplant and non-transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Valid Mono Maintenance</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_THAL_MONO</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Thalidomide monotherapy</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Thalidomide monotherapy. NCCN Other Recommended Regimen for both transplant and non-transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Thalidomide monotherapy (NCCN Other Recommended Regimen for both transplant and non-transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Valid Dual Maintenance</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_BORT_LENA_DUAL</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Bortezomib/lenalidomide dual therapy</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Bortezomib/lenalidomide dual therapy. NCCN Useful in Certain Circumstances for non-transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Bortezomib/lenalidomide dual therapy (NCCN Useful in Certain Circumstances, for non-transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G13" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Valid Dual Maintenance</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_CARF_LENA_DUAL</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Carfilzomib/lenalidomide dual therapy</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Carfilzomib/lenalidomide dual therapy. NCCN Useful in Certain Circumstances for transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Carfilzomib/lenalidomide dual therapy (NCCN Useful in Certain Circumstances for transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr"/>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Valid Dual Maintenance</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_DARA_LENA_DUAL</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Daratumumab/lenalidomide dual therapy</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Daratumumab/lenalidomide dual therapy. NCCN Useful in Certain Circumstances for transplant candidates.</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Daratumumab/lenalidomide dual therapy (NCCN Useful in Certain Circumstances for transplant candidates)'</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G15" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Substitution</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_BORT_IXAZ_SUB</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Bortezomib to ixazomib substitution in maintenance</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Substitution of bortezomib induction therapy for ixazomib as a maintenance therapy does not advance the LOT.</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Substitution of bortezomib induction therapy for ixazomib as a maintenance therapy'</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr"/>
+      <c r="L16" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance End</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_END_RULES</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance regimen end conditions</t>
+        </is>
+      </c>
+      <c r="D17" s="1" t="inlineStr">
+        <is>
+          <t>Once a maintenance regimen has begun (observing valid maintenance medication(s) by itself for at least 120 days), it continues until: (a) discontinuation, (b) presence of an SCT, (c) right censoring (end of follow-up), or (d) the addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.</t>
+        </is>
+      </c>
+      <c r="E17" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Once a maintenance regimen has begun, it continues until discontinuation, presence of an SCT, right censoring (i.e. end of follow-up), or the addition of any non-maintenance MM therapy automatically causes the maintenance regimen to end.'</t>
+        </is>
+      </c>
+      <c r="F17" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G17" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr"/>
+      <c r="L17" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance End</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_REINTRODUCTION_RULE</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>Reintroduction of prior regimen medications ends maintenance</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>The introduction of any MM therapies including therapies that were part of the original regimen does not advance the LOT but ends the maintenance period. Example: a LOT has an initial regimen of Bortezomib+Lenalidomide and later the patient has a Bortezomib mono maintenance regimen; if Lenalidomide restarts then the maintenance regimen will end as 120+ days of only Bortezomib were observed and the reintroduction of Lenalidomide could indicate progression.</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'The introduction of any MM therapies including therapies that were part of the original regimen does not advance the LOT (e.g., a LOT has an initial regimen of Bortezomib+Lenalidomide and later the patient has a Bortezomib mono maintenance regimen; if Lenalidomide restarts at some point then the maintenance regimen will end as we observed 120+ days of only Bortezomib and the reintroduction of Lenalidomide could indicate progression).'</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr"/>
+      <c r="K18" s="1" t="inlineStr"/>
+      <c r="L18" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance End</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>MAINT_END_UNPLANNED_SCT</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>Unplanned SCT ends maintenance</t>
+        </is>
+      </c>
+      <c r="D19" s="1" t="inlineStr">
+        <is>
+          <t>Unplanned SCTs, death, health plan disenrollment, and end of study period all end the maintenance regimen.</t>
+        </is>
+      </c>
+      <c r="E19" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'Unplanned SCTs (defined above), Death, Health plan disenrollment, end of study period' end the maintenance regimen.</t>
+        </is>
+      </c>
+      <c r="F19" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G19" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>NNN</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined but not yet implemented</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr"/>
+      <c r="K19" s="1" t="inlineStr"/>
+      <c r="L19" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Variables</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MAINT_START_DT</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>LOT N maintenance start date</t>
+        </is>
+      </c>
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>Date when the maintenance regimen begins within the LOT. For transition maintenance (situation 1): date when only maintenance medications remain. For post-SCT maintenance (situation 2): first date of valid maintenance therapy within 180 days of the SCT.</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: Maintenance regimen situations 1 and 2 define when maintenance begins within a LOT.</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
+        <is>
+          <t>lot1baseend has LOT1_BASEMAINT_START placeholder</t>
+        </is>
+      </c>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>NNP</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined; partial placeholder in lot1baseend</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr"/>
+      <c r="K20" s="1" t="inlineStr"/>
+      <c r="L20" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Variables</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MAINT_END_DT</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>LOT N maintenance end date</t>
+        </is>
+      </c>
+      <c r="D21" s="1" t="inlineStr">
+        <is>
+          <t>Date when the maintenance regimen ends within the LOT. Ends at: discontinuation, SCT, right censoring, or addition of non-maintenance MM therapy.</t>
+        </is>
+      </c>
+      <c r="E21" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: 'it continues until discontinuation, presence of an SCT, right censoring (i.e. end of follow-up), or the addition of any non-maintenance MM therapy'</t>
+        </is>
+      </c>
+      <c r="F21" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G21" s="1" t="inlineStr">
+        <is>
+          <t>lot1baseend has LOT1_BASEMAINT_END placeholder</t>
+        </is>
+      </c>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>NNP</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined; partial placeholder in lot1baseend</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="inlineStr"/>
+      <c r="K21" s="1" t="inlineStr"/>
+      <c r="L21" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Variables</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MAINT_TYPE</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>LOT N maintenance therapy type</t>
+        </is>
+      </c>
+      <c r="D22" s="1" t="inlineStr">
+        <is>
+          <t>Abbreviation(s) of the maintenance medication(s). Mono: LENA, BORT, DARA, IXAZ, THAL. Dual: BORT+LENA, CARF+LENA, DARA+LENA.</t>
+        </is>
+      </c>
+      <c r="E22" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: Lists all valid mono and dual maintenance therapies.</t>
+        </is>
+      </c>
+      <c r="F22" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G22" s="1" t="inlineStr">
+        <is>
+          <t>lot1baseend has LOT1_BASEMAINT_TYP placeholder</t>
+        </is>
+      </c>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>NNP</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined; partial placeholder in lot1baseend</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr"/>
+      <c r="K22" s="1" t="inlineStr"/>
+      <c r="L22" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>Maintenance Variables</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>LOTN_MAINT_END_REASON</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>LOT N maintenance end reason</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="inlineStr">
+        <is>
+          <t>Categorical: DISCONTINUATION / SCT / CENSORING / NON_MAINT_THERAPY_ADDED / UNPLANNED_SCT / DEATH / DISENROLLMENT / STUDY_END.</t>
+        </is>
+      </c>
+      <c r="E23" s="1" t="inlineStr">
+        <is>
+          <t>Protocol Section 5.1.1: Defines maintenance end conditions.</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>Not yet implemented</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="inlineStr">
+        <is>
+          <t>lot1baseend has LOT1_BASEMAINT_END_REASON placeholder</t>
+        </is>
+      </c>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>NNP</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>Protocol-defined; partial placeholder in lot1baseend</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr"/>
+      <c r="K23" s="1" t="inlineStr"/>
+      <c r="L23" s="1" t="inlineStr">
+        <is>
+          <t>No original spec exists for maintenance</t>
         </is>
       </c>
     </row>

</xml_diff>